<commit_message>
feat: Workshop Floor Plan Editor - Fabric.js canvas with drag/resize/rotate, toolbox, properties panel, save/load layouts, equipment status colors
</commit_message>
<xml_diff>
--- a/人员配置.xlsx
+++ b/人员配置.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$128</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -3765,6 +3768,9 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D128" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>